<commit_message>
increase shotgun stock weight
</commit_message>
<xml_diff>
--- a/changes/shotgun-stocks.xlsx
+++ b/changes/shotgun-stocks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{47705C51-104F-4606-AC94-5FDB3C1F4A5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E9E6B42-103C-4A4F-A446-E2907E2D642E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1905" yWindow="1905" windowWidth="30240" windowHeight="15405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="m4-barrels" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>new</t>
   </si>
@@ -155,13 +155,16 @@
     <t>strength_lessrecoil</t>
   </si>
   <si>
-    <t>agr endcap</t>
-  </si>
-  <si>
     <t>agr buffer</t>
   </si>
   <si>
     <t>agr total endcap</t>
+  </si>
+  <si>
+    <t>agr_870_protection_cap</t>
+  </si>
+  <si>
+    <t>AGR 870</t>
   </si>
 </sst>
 </file>
@@ -1152,10 +1155,10 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="Q3">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R3">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="S3">
         <v>6</v>
@@ -1168,11 +1171,11 @@
       </c>
       <c r="AB3">
         <f>Q3-R3*20-S3*0.8-T3*0.6-V3*5+W3*10+X3/300</f>
-        <v>6</v>
+        <v>3.7999999999999989</v>
       </c>
       <c r="AC3">
         <f t="shared" ref="AC3:AC22" si="2">Q3-R3*20-S3*0.4-T3*0.3-V3*5+W3*10+X3/300</f>
-        <v>10.199999999999999</v>
+        <v>7.9999999999999991</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.25">
@@ -1209,7 +1212,7 @@
         <v>22</v>
       </c>
       <c r="R4">
-        <v>0.24</v>
+        <v>0.34</v>
       </c>
       <c r="S4">
         <v>-9</v>
@@ -1222,11 +1225,11 @@
       </c>
       <c r="AB4">
         <f t="shared" ref="AB4:AB22" si="4">Q4-R4*20-S4*0.8-T4*0.6-V4*5+W4*10+X4/300</f>
-        <v>29.2</v>
+        <v>27.2</v>
       </c>
       <c r="AC4">
         <f t="shared" si="2"/>
-        <v>23.2</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
@@ -1263,7 +1266,7 @@
       </c>
       <c r="R5">
         <f t="shared" ref="R5:T5" si="6">R12+R22</f>
-        <v>0.26</v>
+        <v>0.36</v>
       </c>
       <c r="S5">
         <f t="shared" si="6"/>
@@ -1275,11 +1278,11 @@
       </c>
       <c r="AB5">
         <f t="shared" si="4"/>
-        <v>28.8</v>
+        <v>26.8</v>
       </c>
       <c r="AC5">
         <f t="shared" si="2"/>
-        <v>23.3</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.25">
@@ -1319,7 +1322,7 @@
       </c>
       <c r="R6">
         <f>R13+R18+R19</f>
-        <v>0.42000000000000004</v>
+        <v>0.44999999999999996</v>
       </c>
       <c r="S6">
         <f>S13+S18+S19</f>
@@ -1327,7 +1330,7 @@
       </c>
       <c r="T6">
         <f>T13+T18+T19</f>
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="AA6">
         <v>1000</v>
@@ -1338,12 +1341,12 @@
       </c>
       <c r="AC6">
         <f t="shared" si="2"/>
-        <v>19.600000000000001</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7">
         <f>C14+C20</f>
@@ -1374,15 +1377,15 @@
       </c>
       <c r="Q7">
         <f>Q14+Q20</f>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R7">
         <f t="shared" ref="R7:T7" si="8">R14+R20</f>
-        <v>0.13999999999999999</v>
+        <v>0.19</v>
       </c>
       <c r="S7">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T7">
         <f t="shared" si="8"/>
@@ -1390,11 +1393,11 @@
       </c>
       <c r="AB7">
         <f t="shared" si="4"/>
-        <v>8.6</v>
+        <v>4.7999999999999989</v>
       </c>
       <c r="AC7">
         <f t="shared" si="2"/>
-        <v>11.4</v>
+        <v>7.9999999999999991</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.25">
@@ -1431,11 +1434,11 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:T8" si="10">R14+R18+R21</f>
-        <v>0.38</v>
+        <v>0.43000000000000005</v>
       </c>
       <c r="S8">
         <f t="shared" si="10"/>
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T8">
         <f t="shared" si="10"/>
@@ -1443,11 +1446,11 @@
       </c>
       <c r="AB8">
         <f t="shared" si="4"/>
-        <v>28.400000000000002</v>
+        <v>26.599999999999998</v>
       </c>
       <c r="AC8">
         <f t="shared" si="2"/>
-        <v>20.399999999999999</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.25">
@@ -1484,7 +1487,7 @@
         <v>19</v>
       </c>
       <c r="R9">
-        <v>0.28999999999999998</v>
+        <v>0.38</v>
       </c>
       <c r="S9">
         <v>-12</v>
@@ -1496,12 +1499,12 @@
         <v>1000</v>
       </c>
       <c r="AB9">
-        <f>Q9-R9*20-S9*0.8-T9*0.6-V9*5+W9*10+X9/300</f>
-        <v>31.8</v>
+        <f t="shared" si="4"/>
+        <v>30</v>
       </c>
       <c r="AC9">
         <f>Q9-R9*20-S9*0.4-T9*0.3-V9*5+W9*10+X9/300</f>
-        <v>22.5</v>
+        <v>20.700000000000003</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.25">
@@ -1541,7 +1544,7 @@
       </c>
       <c r="R10">
         <f>R15+R16</f>
-        <v>0.24000000000000002</v>
+        <v>0.32</v>
       </c>
       <c r="S10">
         <f>S15+S16</f>
@@ -1556,11 +1559,11 @@
       </c>
       <c r="AB10">
         <f t="shared" si="4"/>
-        <v>32</v>
+        <v>30.4</v>
       </c>
       <c r="AC10">
         <f t="shared" si="2"/>
-        <v>22.599999999999998</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.25">
@@ -1615,7 +1618,7 @@
         <v>22</v>
       </c>
       <c r="R12">
-        <v>0.22</v>
+        <v>0.32</v>
       </c>
       <c r="S12">
         <v>-7</v>
@@ -1628,11 +1631,11 @@
       </c>
       <c r="AB12">
         <f t="shared" si="4"/>
-        <v>28.6</v>
+        <v>26.599999999999998</v>
       </c>
       <c r="AC12">
         <f t="shared" si="2"/>
-        <v>23.1</v>
+        <v>21.099999999999998</v>
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.25">
@@ -1669,13 +1672,13 @@
         <v>-7</v>
       </c>
       <c r="R13">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="S13">
         <v>-1</v>
       </c>
       <c r="T13">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AA13">
         <v>1000</v>
@@ -1686,7 +1689,7 @@
       </c>
       <c r="AC13">
         <f t="shared" si="2"/>
-        <v>-9.6999999999999993</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.25">
@@ -1723,10 +1726,10 @@
         <v>1</v>
       </c>
       <c r="R14">
-        <v>0.12</v>
+        <v>0.17</v>
       </c>
       <c r="S14">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T14">
         <v>-4</v>
@@ -1736,11 +1739,11 @@
       </c>
       <c r="AB14">
         <f t="shared" si="4"/>
-        <v>4.2</v>
+        <v>2.4</v>
       </c>
       <c r="AC14">
         <f t="shared" si="2"/>
-        <v>1.4000000000000001</v>
+        <v>-2.2204460492503131E-16</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.25">
@@ -1777,7 +1780,7 @@
         <v>16</v>
       </c>
       <c r="R15">
-        <v>0.2</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="S15">
         <v>-13</v>
@@ -1790,11 +1793,11 @@
       </c>
       <c r="AB15">
         <f t="shared" si="4"/>
-        <v>30.799999999999997</v>
+        <v>29.199999999999996</v>
       </c>
       <c r="AC15">
         <f t="shared" si="2"/>
-        <v>21.4</v>
+        <v>19.799999999999997</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.25">
@@ -1963,29 +1966,27 @@
       </c>
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="1">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20">
         <v>16</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20">
         <v>0.02</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20">
         <v>8</v>
       </c>
-      <c r="F20" s="1">
+      <c r="F20">
         <v>8</v>
       </c>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
+      <c r="M20">
+        <v>100</v>
+      </c>
       <c r="N20">
         <f t="shared" si="3"/>
         <v>4.3999999999999995</v>
@@ -1994,38 +1995,34 @@
         <f t="shared" si="1"/>
         <v>9.9999999999999982</v>
       </c>
-      <c r="Q20" s="1">
-        <v>16</v>
-      </c>
-      <c r="R20" s="1">
+      <c r="Q20">
+        <v>14</v>
+      </c>
+      <c r="R20">
         <v>0.02</v>
       </c>
-      <c r="S20" s="1">
+      <c r="S20">
         <v>8</v>
       </c>
-      <c r="T20" s="1">
+      <c r="T20">
         <v>8</v>
       </c>
-      <c r="U20" s="1"/>
-      <c r="V20" s="1"/>
-      <c r="W20" s="1"/>
-      <c r="X20" s="1"/>
-      <c r="Y20" s="1"/>
-      <c r="Z20" s="1"/>
-      <c r="AA20" s="1"/>
+      <c r="AA20">
+        <v>100</v>
+      </c>
       <c r="AB20">
         <f t="shared" si="4"/>
-        <v>4.3999999999999995</v>
+        <v>2.3999999999999995</v>
       </c>
       <c r="AC20">
         <f t="shared" si="2"/>
-        <v>9.9999999999999982</v>
+        <v>7.9999999999999982</v>
       </c>
     </row>
     <row r="21" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" s="1">
         <v>0</v>
@@ -2057,6 +2054,10 @@
       <c r="Y21" s="1"/>
       <c r="Z21" s="1"/>
       <c r="AA21" s="1"/>
+      <c r="AB21">
+        <f t="shared" si="4"/>
+        <v>-2</v>
+      </c>
     </row>
     <row r="22" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>

</xml_diff>